<commit_message>
Ship Ver 1.3.8: split limit rows, batch TR print, and photo zoom.
Replace the single 限值 expression with 上限/下限 numbers, keep custom card names unless the first standard changes, and let testers pick local vs share when opening the project folder.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/data_tables/5点法.xlsx
+++ b/templates/data_tables/5点法.xlsx
@@ -1,78 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ikaruga/Desktop/Reach/report creator/templates/data_tables/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBA391EC-91CE-1C44-B5A3-EC9712639581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17340" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
-  <si>
-    <t>-40°C</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>25°C</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>85°C</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>9V</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>14V</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>16V</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>限值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="新細明體"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="新細明體"/>
+      <charset val="136"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="新細明體"/>
-      <family val="3"/>
-      <charset val="136"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -90,32 +52,94 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -403,73 +427,110 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="19.59765625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="10" width="11" style="3" customWidth="1"/>
-    <col min="11" max="16384" width="9" style="1"/>
+    <col width="19.59765625" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
+    <col width="11" customWidth="1" style="4" min="2" max="10"/>
+    <col width="9" customWidth="1" style="1" min="11" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>样品编号
+Sample No.</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>-40°C</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>25°C</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>85°C</t>
+        </is>
+      </c>
     </row>
-    <row r="2" spans="1:10" ht="15">
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>5</v>
+    <row r="2" ht="15" customHeight="1">
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>9V</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>14V</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>16V</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>9V</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>14V</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>16V</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>9V</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>14V</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>16V</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="1" t="s">
-        <v>6</v>
+    <row r="3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>上限</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>下限</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:J1"/>
+  <mergeCells count="4">
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="A1:A4"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="I1:K1"/>
   </mergeCells>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>